<commit_message>
Décisions : import mensuel finance Octobre 2026 (13 Oui, 2 Non, mémoire créée)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KigtzPVpDSdWiBfvZW9e6r
</commit_message>
<xml_diff>
--- a/outputs/import-mensuel-finance/runs/Database XBH Octobre 2026 v2.xlsx
+++ b/outputs/import-mensuel-finance/runs/Database XBH Octobre 2026 v2.xlsx
@@ -3337,18 +3337,6 @@
           <t>Italie</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>1850959.06</v>
-      </c>
-      <c r="G76" t="n">
-        <v>1825513.5</v>
-      </c>
-      <c r="H76" t="n">
-        <v>1301598.3</v>
-      </c>
-      <c r="I76" t="n">
-        <v>4451</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -14242,18 +14230,6 @@
         <is>
           <t>Argentine</t>
         </is>
-      </c>
-      <c r="F359" t="n">
-        <v>5546505.1</v>
-      </c>
-      <c r="G359" t="n">
-        <v>5292208.99</v>
-      </c>
-      <c r="H359" t="n">
-        <v>3471600.13</v>
-      </c>
-      <c r="I359" t="n">
-        <v>926</v>
       </c>
     </row>
     <row r="360">
@@ -15893,7 +15869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16857,6 +16833,94 @@
       <c r="D34" t="inlineStr">
         <is>
           <t>(b) absent du fichier finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>155</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>FH.X8BS2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>(g) correspondance rejetée (proposée avec FH.X87S2)</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>5546505.1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5292208.99</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3471600.13</v>
+      </c>
+      <c r="H35" t="n">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>database l.359</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FH.X87S2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>(b) absent du fichier finance (après rejet de FH.X8BS2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>303</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FB.VXVFM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>(g) correspondance rejetée (proposée avec FH.XVVFM)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1850959.06</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1825513.5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1301598.3</v>
+      </c>
+      <c r="H37" t="n">
+        <v>4451</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>database l.76</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FH.XVVFM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>(b) absent du fichier finance (après rejet de FB.VXVFM)</t>
         </is>
       </c>
     </row>
@@ -16935,9 +16999,14 @@
       <c r="D2" t="n">
         <v>0.5</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -16966,9 +17035,14 @@
       <c r="D3" t="n">
         <v>0.5</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -16997,9 +17071,14 @@
       <c r="D4" t="n">
         <v>0.5</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -17028,9 +17107,14 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Rejetée le 2026-10-28</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -17059,9 +17143,14 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -17090,9 +17179,14 @@
       <c r="D7" t="n">
         <v>0.5</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -17121,9 +17215,14 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -17152,9 +17251,14 @@
       <c r="D9" t="n">
         <v>0.5</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -17183,9 +17287,14 @@
       <c r="D10" t="n">
         <v>0.5</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -17214,9 +17323,14 @@
       <c r="D11" t="n">
         <v>0.5</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -17245,9 +17359,14 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Rejetée le 2026-10-28</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -17276,9 +17395,14 @@
       <c r="D13" t="n">
         <v>1</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -17307,9 +17431,14 @@
       <c r="D14" t="n">
         <v>0.5</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -17338,9 +17467,14 @@
       <c r="D15" t="n">
         <v>0.5</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -17369,9 +17503,14 @@
       <c r="D16" t="n">
         <v>0.5</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>En attente de confirmation</t>
+          <t>Confirmée le 2026-10-28 (certaine)</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -17392,7 +17531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17450,13 +17589,13 @@
         <v>1516914829.77</v>
       </c>
       <c r="D2" t="n">
-        <v>1467184114.25</v>
+        <v>1459786650.09</v>
       </c>
       <c r="E2" t="n">
-        <v>49730715.52</v>
+        <v>57128179.68</v>
       </c>
       <c r="F2" t="n">
-        <v>62990146.13</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -17480,13 +17619,13 @@
         <v>1463742453.74</v>
       </c>
       <c r="D3" t="n">
-        <v>1416332660.37</v>
+        <v>1409214937.88</v>
       </c>
       <c r="E3" t="n">
-        <v>47409793.37</v>
+        <v>54527515.86</v>
       </c>
       <c r="F3" t="n">
-        <v>60628959.79</v>
+        <v>-0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -17510,13 +17649,13 @@
         <v>1092766728.71</v>
       </c>
       <c r="D4" t="n">
-        <v>1059643928.11</v>
+        <v>1054870729.68</v>
       </c>
       <c r="E4" t="n">
-        <v>33122800.6</v>
+        <v>37895999.03</v>
       </c>
       <c r="F4" t="n">
-        <v>46181445.83</v>
+        <v>-0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -17540,13 +17679,13 @@
         <v>1801640</v>
       </c>
       <c r="D5" t="n">
-        <v>1760223</v>
+        <v>1754846</v>
       </c>
       <c r="E5" t="n">
-        <v>41417</v>
+        <v>46794</v>
       </c>
       <c r="F5" t="n">
-        <v>46477</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -17557,6 +17696,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -17564,7 +17704,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>370</v>
+        <v>383</v>
       </c>
     </row>
     <row r="8">
@@ -17574,7 +17714,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -17584,7 +17724,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -17604,7 +17744,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -17617,6 +17757,7 @@
         <v>398</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -17675,6 +17816,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -17683,8 +17825,50 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>indisponible : décisions à prendre</t>
-        </is>
+          <t>possible (case à cocher par Baptiste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Prise en compte des décisions</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Décisions « Oui »</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Décisions « Non »</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Décisions manquantes</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>